<commit_message>
feat(proto): 完善 proto 文件生成
</commit_message>
<xml_diff>
--- a/assets/xls/基础类型.xlsx
+++ b/assets/xls/基础类型.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="21315" windowHeight="10680" tabRatio="535"/>
+    <workbookView windowWidth="21555" windowHeight="11265" tabRatio="535"/>
   </bookViews>
   <sheets>
     <sheet name="Resource" sheetId="7" r:id="rId1"/>
@@ -36,7 +36,7 @@
     <t>ID</t>
   </si>
   <si>
-    <t>Count</t>
+    <t>Amount</t>
   </si>
   <si>
     <t>int32</t>

</xml_diff>